<commit_message>
Fix Gestisci: le aggiunte non vengono più scritte sul file xlsx di default
- save_file_editor: rimossa scrittura su xlsx, ticker estratti dalle righe del DataTable
- Al refresh della pagina, Gestisci mostra sempre solo i ticker del file di default
- Files/ETF.xlsx: rimosso BMPS.MI rimasto dal vecchio codice

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Files/ETF.xlsx
+++ b/Files/ETF.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>

</xml_diff>